<commit_message>
CCTP-14276 - capture action import/export (#721)
* import/export capture action progress

* capture import/export updates after merge

* add new columns to test spreadsheets

* add capture case for batch create

* include capture in batch create

* fix existing tests for capture action

* feat(Capture -> Export): Add `captureTimeout` field in Capture Action

* feat(Capture -> DataGrid): Render `captureTimeout` field in Main DataGrid

* feat(Capture -> Preview Modal): Render `captureTimeout` field in Preview Modal

* fix: Resolve test case failures

* add capture action import test

* rename interface

---------

Co-authored-by: Bhopal Singh <bhopal.singh@libertymutual.com>
</commit_message>
<xml_diff>
--- a/src/components/tabs/dynamicCallFlow/action/Xlsx/test/AISGMain-redirect-url-invalid.xlsx
+++ b/src/components/tabs/dynamicCallFlow/action/Xlsx/test/AISGMain-redirect-url-invalid.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\n0354604\IdeaProjects\cicct-softphone-admin-ui-merge-refactor\src\components\tabs\dynamicCallFlow\action\Xlsx\test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n1584945/repos/cicct/cicct-softphone-admin-ui/src/components/tabs/dynamicCallFlow/action/Xlsx/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86BDC70B-E7A2-47ED-8777-ADE875C61C72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3A78606-CB8A-5647-8B4C-77EE60FD3199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="960" yWindow="500" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1 - dynamic-flow-17150001" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="61">
   <si>
     <t>actionId</t>
   </si>
@@ -195,12 +195,27 @@
   <si>
     <t>24io23</t>
   </si>
+  <si>
+    <t>captureValidLengths</t>
+  </si>
+  <si>
+    <t>captureEndpoint</t>
+  </si>
+  <si>
+    <t>captureParameter</t>
+  </si>
+  <si>
+    <t>captureTimeout</t>
+  </si>
+  <si>
+    <t>captureOutcomes</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -229,6 +244,13 @@
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
       <name val="Helvetica Neue"/>
       <family val="2"/>
     </font>
@@ -414,12 +436,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -489,8 +514,12 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1649,35 +1678,36 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:JD23"/>
-  <sheetFormatPr defaultColWidth="8.28515625" defaultRowHeight="20.100000000000001" customHeight="1"/>
+  <dimension ref="A1:JI23"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.33203125" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="33.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="34.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="31.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="24.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="27.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="33.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="34.33203125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="31.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="24.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="27.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.83203125" style="1" customWidth="1"/>
     <col min="17" max="17" width="27" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="24.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="31.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="25.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="23" max="264" width="8.28515625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="24.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="31.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="25.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="26" width="11.33203125" style="1" customWidth="1"/>
+    <col min="27" max="27" width="11.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="269" width="8.33203125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="20.25" customHeight="1">
+    <row r="1" spans="1:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1741,9 +1771,24 @@
       <c r="U1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="V1" s="2"/>
+      <c r="V1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA1" s="2"/>
     </row>
-    <row r="2" spans="1:22" ht="20.25" customHeight="1">
+    <row r="2" spans="1:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="3" t="s">
         <v>17</v>
       </c>
@@ -1775,8 +1820,13 @@
       <c r="T2" s="6"/>
       <c r="U2" s="7"/>
       <c r="V2" s="7"/>
+      <c r="W2" s="7"/>
+      <c r="X2" s="7"/>
+      <c r="Y2" s="7"/>
+      <c r="Z2" s="7"/>
+      <c r="AA2" s="7"/>
     </row>
-    <row r="3" spans="1:22" ht="20.100000000000001" customHeight="1">
+    <row r="3" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="8" t="s">
         <v>18</v>
       </c>
@@ -1811,8 +1861,13 @@
       <c r="T3" s="11"/>
       <c r="U3" s="12"/>
       <c r="V3" s="12"/>
+      <c r="W3" s="12"/>
+      <c r="X3" s="12"/>
+      <c r="Y3" s="12"/>
+      <c r="Z3" s="12"/>
+      <c r="AA3" s="12"/>
     </row>
-    <row r="4" spans="1:22" ht="20.100000000000001" customHeight="1">
+    <row r="4" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="8" t="s">
         <v>19</v>
       </c>
@@ -1847,8 +1902,13 @@
       <c r="T4" s="11"/>
       <c r="U4" s="12"/>
       <c r="V4" s="12"/>
+      <c r="W4" s="12"/>
+      <c r="X4" s="12"/>
+      <c r="Y4" s="12"/>
+      <c r="Z4" s="12"/>
+      <c r="AA4" s="12"/>
     </row>
-    <row r="5" spans="1:22" ht="20.100000000000001" customHeight="1">
+    <row r="5" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="8" t="s">
         <v>20</v>
       </c>
@@ -1883,8 +1943,13 @@
       <c r="T5" s="11"/>
       <c r="U5" s="12"/>
       <c r="V5" s="12"/>
+      <c r="W5" s="12"/>
+      <c r="X5" s="12"/>
+      <c r="Y5" s="12"/>
+      <c r="Z5" s="12"/>
+      <c r="AA5" s="12"/>
     </row>
-    <row r="6" spans="1:22" ht="95.1" customHeight="1">
+    <row r="6" spans="1:27" ht="95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="8" t="s">
         <v>53</v>
       </c>
@@ -1933,8 +1998,13 @@
       <c r="T6" s="11"/>
       <c r="U6" s="12"/>
       <c r="V6" s="12"/>
+      <c r="W6" s="12"/>
+      <c r="X6" s="12"/>
+      <c r="Y6" s="12"/>
+      <c r="Z6" s="12"/>
+      <c r="AA6" s="12"/>
     </row>
-    <row r="7" spans="1:22" ht="20.100000000000001" customHeight="1">
+    <row r="7" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="8" t="s">
         <v>21</v>
       </c>
@@ -1973,8 +2043,13 @@
       </c>
       <c r="U7" s="12"/>
       <c r="V7" s="12"/>
+      <c r="W7" s="12"/>
+      <c r="X7" s="12"/>
+      <c r="Y7" s="12"/>
+      <c r="Z7" s="12"/>
+      <c r="AA7" s="12"/>
     </row>
-    <row r="8" spans="1:22" ht="20.100000000000001" customHeight="1">
+    <row r="8" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="8" t="s">
         <v>21</v>
       </c>
@@ -2011,8 +2086,13 @@
       </c>
       <c r="U8" s="12"/>
       <c r="V8" s="12"/>
+      <c r="W8" s="12"/>
+      <c r="X8" s="12"/>
+      <c r="Y8" s="12"/>
+      <c r="Z8" s="12"/>
+      <c r="AA8" s="12"/>
     </row>
-    <row r="9" spans="1:22" ht="20.100000000000001" customHeight="1">
+    <row r="9" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="8" t="s">
         <v>21</v>
       </c>
@@ -2049,8 +2129,13 @@
       </c>
       <c r="U9" s="12"/>
       <c r="V9" s="12"/>
+      <c r="W9" s="12"/>
+      <c r="X9" s="12"/>
+      <c r="Y9" s="12"/>
+      <c r="Z9" s="12"/>
+      <c r="AA9" s="12"/>
     </row>
-    <row r="10" spans="1:22" ht="20.100000000000001" customHeight="1">
+    <row r="10" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="8" t="s">
         <v>21</v>
       </c>
@@ -2087,8 +2172,13 @@
       </c>
       <c r="U10" s="12"/>
       <c r="V10" s="12"/>
+      <c r="W10" s="12"/>
+      <c r="X10" s="12"/>
+      <c r="Y10" s="12"/>
+      <c r="Z10" s="12"/>
+      <c r="AA10" s="12"/>
     </row>
-    <row r="11" spans="1:22" ht="20.100000000000001" customHeight="1">
+    <row r="11" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="8" t="s">
         <v>21</v>
       </c>
@@ -2123,8 +2213,13 @@
       <c r="T11" s="15"/>
       <c r="U11" s="12"/>
       <c r="V11" s="12"/>
+      <c r="W11" s="12"/>
+      <c r="X11" s="12"/>
+      <c r="Y11" s="12"/>
+      <c r="Z11" s="12"/>
+      <c r="AA11" s="12"/>
     </row>
-    <row r="12" spans="1:22" ht="20.100000000000001" customHeight="1">
+    <row r="12" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="8" t="s">
         <v>21</v>
       </c>
@@ -2159,8 +2254,13 @@
       <c r="T12" s="15"/>
       <c r="U12" s="12"/>
       <c r="V12" s="12"/>
+      <c r="W12" s="12"/>
+      <c r="X12" s="12"/>
+      <c r="Y12" s="12"/>
+      <c r="Z12" s="12"/>
+      <c r="AA12" s="12"/>
     </row>
-    <row r="13" spans="1:22" ht="25.5">
+    <row r="13" spans="1:27" ht="28" x14ac:dyDescent="0.15">
       <c r="A13" s="8" t="s">
         <v>15</v>
       </c>
@@ -2209,8 +2309,13 @@
       <c r="T13" s="11"/>
       <c r="U13" s="12"/>
       <c r="V13" s="12"/>
+      <c r="W13" s="12"/>
+      <c r="X13" s="12"/>
+      <c r="Y13" s="12"/>
+      <c r="Z13" s="12"/>
+      <c r="AA13" s="12"/>
     </row>
-    <row r="14" spans="1:22" ht="20.100000000000001" customHeight="1">
+    <row r="14" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="8" t="s">
         <v>22</v>
       </c>
@@ -2247,8 +2352,13 @@
       </c>
       <c r="U14" s="12"/>
       <c r="V14" s="12"/>
+      <c r="W14" s="12"/>
+      <c r="X14" s="12"/>
+      <c r="Y14" s="12"/>
+      <c r="Z14" s="12"/>
+      <c r="AA14" s="12"/>
     </row>
-    <row r="15" spans="1:22" ht="20.100000000000001" customHeight="1">
+    <row r="15" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="8" t="s">
         <v>22</v>
       </c>
@@ -2285,8 +2395,13 @@
       </c>
       <c r="U15" s="12"/>
       <c r="V15" s="12"/>
+      <c r="W15" s="12"/>
+      <c r="X15" s="12"/>
+      <c r="Y15" s="12"/>
+      <c r="Z15" s="12"/>
+      <c r="AA15" s="12"/>
     </row>
-    <row r="16" spans="1:22" ht="20.100000000000001" customHeight="1">
+    <row r="16" spans="1:27" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="8" t="s">
         <v>22</v>
       </c>
@@ -2321,8 +2436,13 @@
       <c r="T16" s="15"/>
       <c r="U16" s="12"/>
       <c r="V16" s="12"/>
+      <c r="W16" s="12"/>
+      <c r="X16" s="12"/>
+      <c r="Y16" s="12"/>
+      <c r="Z16" s="12"/>
+      <c r="AA16" s="12"/>
     </row>
-    <row r="17" spans="1:264" ht="20.100000000000001" customHeight="1">
+    <row r="17" spans="1:269" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="8" t="s">
         <v>22</v>
       </c>
@@ -2357,8 +2477,13 @@
       <c r="T17" s="15"/>
       <c r="U17" s="12"/>
       <c r="V17" s="12"/>
+      <c r="W17" s="12"/>
+      <c r="X17" s="12"/>
+      <c r="Y17" s="12"/>
+      <c r="Z17" s="12"/>
+      <c r="AA17" s="12"/>
     </row>
-    <row r="18" spans="1:264" ht="25.5">
+    <row r="18" spans="1:269" ht="28" x14ac:dyDescent="0.15">
       <c r="A18" s="8" t="s">
         <v>16</v>
       </c>
@@ -2407,8 +2532,13 @@
       <c r="T18" s="22"/>
       <c r="U18" s="12"/>
       <c r="V18" s="12"/>
+      <c r="W18" s="12"/>
+      <c r="X18" s="12"/>
+      <c r="Y18" s="12"/>
+      <c r="Z18" s="12"/>
+      <c r="AA18" s="12"/>
     </row>
-    <row r="19" spans="1:264" ht="20.100000000000001" customHeight="1">
+    <row r="19" spans="1:269" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="8" t="s">
         <v>23</v>
       </c>
@@ -2445,8 +2575,13 @@
       </c>
       <c r="U19" s="12"/>
       <c r="V19" s="12"/>
+      <c r="W19" s="12"/>
+      <c r="X19" s="12"/>
+      <c r="Y19" s="12"/>
+      <c r="Z19" s="12"/>
+      <c r="AA19" s="12"/>
     </row>
-    <row r="20" spans="1:264" ht="20.100000000000001" customHeight="1">
+    <row r="20" spans="1:269" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="8" t="s">
         <v>23</v>
       </c>
@@ -2483,8 +2618,13 @@
       </c>
       <c r="U20" s="12"/>
       <c r="V20" s="12"/>
+      <c r="W20" s="12"/>
+      <c r="X20" s="12"/>
+      <c r="Y20" s="12"/>
+      <c r="Z20" s="12"/>
+      <c r="AA20" s="12"/>
     </row>
-    <row r="21" spans="1:264" ht="20.100000000000001" customHeight="1">
+    <row r="21" spans="1:269" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="8" t="s">
         <v>23</v>
       </c>
@@ -2519,8 +2659,13 @@
       <c r="T21" s="15"/>
       <c r="U21" s="12"/>
       <c r="V21" s="12"/>
+      <c r="W21" s="12"/>
+      <c r="X21" s="12"/>
+      <c r="Y21" s="12"/>
+      <c r="Z21" s="12"/>
+      <c r="AA21" s="12"/>
     </row>
-    <row r="22" spans="1:264" ht="20.100000000000001" customHeight="1">
+    <row r="22" spans="1:269" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="16" t="s">
         <v>23</v>
       </c>
@@ -2555,11 +2700,11 @@
       <c r="T22" s="17"/>
       <c r="U22" s="19"/>
       <c r="V22" s="19"/>
-      <c r="W22" s="20"/>
-      <c r="X22" s="20"/>
-      <c r="Y22" s="20"/>
-      <c r="Z22" s="20"/>
-      <c r="AA22" s="20"/>
+      <c r="W22" s="19"/>
+      <c r="X22" s="19"/>
+      <c r="Y22" s="19"/>
+      <c r="Z22" s="19"/>
+      <c r="AA22" s="19"/>
       <c r="AB22" s="20"/>
       <c r="AC22" s="20"/>
       <c r="AD22" s="20"/>
@@ -2797,8 +2942,13 @@
       <c r="JB22" s="20"/>
       <c r="JC22" s="20"/>
       <c r="JD22" s="20"/>
+      <c r="JE22" s="20"/>
+      <c r="JF22" s="20"/>
+      <c r="JG22" s="20"/>
+      <c r="JH22" s="20"/>
+      <c r="JI22" s="20"/>
     </row>
-    <row r="23" spans="1:264" ht="20.100000000000001" customHeight="1">
+    <row r="23" spans="1:269" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="1">
         <v>8</v>
       </c>
@@ -2808,6 +2958,11 @@
       <c r="U23" s="1" t="s">
         <v>55</v>
       </c>
+      <c r="V23" s="23"/>
+      <c r="W23" s="23"/>
+      <c r="X23" s="23"/>
+      <c r="Y23" s="23"/>
+      <c r="Z23" s="23"/>
     </row>
   </sheetData>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>

</xml_diff>